<commit_message>
Admin direct reportee testcase half completed
</commit_message>
<xml_diff>
--- a/testData/testdata.xlsx
+++ b/testData/testdata.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="57">
   <si>
     <t>Product Name</t>
   </si>
@@ -298,7 +298,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -307,6 +307,24 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
@@ -760,7 +778,7 @@
         <v>23</v>
       </c>
       <c r="B2" s="4"/>
-      <c r="E2" t="s" s="18">
+      <c r="E2" t="s" s="36">
         <v>55</v>
       </c>
     </row>
@@ -771,7 +789,7 @@
       <c r="B3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E3" t="s" s="19">
+      <c r="E3" t="s" s="37">
         <v>55</v>
       </c>
     </row>
@@ -785,7 +803,7 @@
       <c r="C4" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="E4" t="s" s="20">
+      <c r="E4" t="s" s="38">
         <v>55</v>
       </c>
     </row>
@@ -794,7 +812,7 @@
       <c r="C5" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="E5" t="s" s="21">
+      <c r="E5" t="s" s="39">
         <v>55</v>
       </c>
     </row>
@@ -802,7 +820,7 @@
       <c r="B6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E6" t="s" s="22">
+      <c r="E6" t="s" s="40">
         <v>55</v>
       </c>
     </row>
@@ -827,7 +845,7 @@
       <c r="C8" t="s" s="0">
         <v>25</v>
       </c>
-      <c r="E8" t="s" s="25">
+      <c r="E8" t="s" s="43">
         <v>56</v>
       </c>
     </row>

</xml_diff>

<commit_message>
pointsDistribution direct deportees Add points not yet completed
</commit_message>
<xml_diff>
--- a/testData/testdata.xlsx
+++ b/testData/testdata.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28627"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28723"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EEF1AA93-1FDA-41D6-96B3-6151ABAE3FAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0CE7046C-B6F7-4966-9497-6A697DF6BA80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -13,10 +13,11 @@
     <sheet name="CheerUpBuddySendBadgeForm" sheetId="3" r:id="rId3"/>
     <sheet name="Badges " sheetId="4" r:id="rId4"/>
     <sheet name="Earn" sheetId="5" r:id="rId5"/>
+    <sheet name="pointsDistributionFilterNames" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="68">
   <si>
     <t>Product Name</t>
   </si>
@@ -202,18 +203,50 @@
     <t>(//p[text()='Wellness'])[1]</t>
   </si>
   <si>
-    <t>Passed</t>
-  </si>
-  <si>
-    <t>Failed</t>
+    <t>BU Name</t>
+  </si>
+  <si>
+    <t>Add Points Category</t>
+  </si>
+  <si>
+    <t>All Business Units</t>
+  </si>
+  <si>
+    <t>Distribute</t>
+  </si>
+  <si>
+    <t>ACS</t>
+  </si>
+  <si>
+    <t>Award</t>
+  </si>
+  <si>
+    <t>DATA</t>
+  </si>
+  <si>
+    <t>DEX</t>
+  </si>
+  <si>
+    <t>IOT</t>
+  </si>
+  <si>
+    <t>ILD</t>
+  </si>
+  <si>
+    <t>SIMS</t>
+  </si>
+  <si>
+    <t>RSBW</t>
+  </si>
+  <si>
+    <t>SALESFORCE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -244,8 +277,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -264,26 +304,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="none">
-        <bgColor indexed="17"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <bgColor indexed="17"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="none">
-        <bgColor indexed="10"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <bgColor indexed="10"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -298,51 +318,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="true"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="true"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -627,7 +610,7 @@
   <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="56.85546875"/>
+    <col min="1" max="1" width="56.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15.75">
@@ -639,52 +622,52 @@
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" t="s" s="0">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" t="s" s="0">
+      <c r="A7" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" t="s" s="0">
+      <c r="A8" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" t="s" s="0">
+      <c r="A9" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" t="s" s="0">
+      <c r="A10" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" t="s" s="0">
+      <c r="A11" t="s">
         <v>10</v>
       </c>
     </row>
@@ -698,13 +681,13 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="24.42578125"/>
-    <col min="2" max="2" customWidth="true" width="28.28515625"/>
-    <col min="3" max="3" customWidth="true" width="25.5703125"/>
-    <col min="4" max="4" customWidth="true" width="16.5703125"/>
-    <col min="5" max="5" customWidth="true" width="17.0"/>
-    <col min="6" max="6" customWidth="true" width="14.0"/>
-    <col min="7" max="7" customWidth="true" width="17.28515625"/>
+    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="2" max="2" width="28.28515625" customWidth="1"/>
+    <col min="3" max="3" width="25.5703125" customWidth="1"/>
+    <col min="4" max="4" width="16.5703125" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="17.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -716,26 +699,26 @@
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>13</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>15</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>16</v>
       </c>
     </row>
@@ -749,11 +732,11 @@
   <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="41.28515625"/>
-    <col min="2" max="2" customWidth="true" width="38.28515625"/>
-    <col min="3" max="3" customWidth="true" width="32.5703125"/>
-    <col min="4" max="4" customWidth="true" width="31.42578125"/>
-    <col min="5" max="5" customWidth="true" width="32.42578125"/>
+    <col min="1" max="1" width="41.28515625" customWidth="1"/>
+    <col min="2" max="2" width="38.28515625" customWidth="1"/>
+    <col min="3" max="3" width="32.5703125" customWidth="1"/>
+    <col min="4" max="4" width="31.42578125" customWidth="1"/>
+    <col min="5" max="5" width="32.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -778,9 +761,6 @@
         <v>23</v>
       </c>
       <c r="B2" s="4"/>
-      <c r="E2" t="s" s="36">
-        <v>55</v>
-      </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="4" t="s">
@@ -789,9 +769,6 @@
       <c r="B3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E3" t="s" s="37">
-        <v>55</v>
-      </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="4" t="s">
@@ -800,29 +777,20 @@
       <c r="B4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" t="s" s="0">
+      <c r="C4" t="s">
         <v>25</v>
-      </c>
-      <c r="E4" t="s" s="38">
-        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="B5" s="4"/>
-      <c r="C5" t="s" s="0">
+      <c r="C5" t="s">
         <v>25</v>
-      </c>
-      <c r="E5" t="s" s="39">
-        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="B6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E6" t="s" s="40">
-        <v>55</v>
-      </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="4" t="s">
@@ -831,7 +799,7 @@
       <c r="B7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C7" t="s" s="0">
+      <c r="C7" t="s">
         <v>25</v>
       </c>
     </row>
@@ -842,11 +810,8 @@
       <c r="B8" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C8" t="s" s="0">
+      <c r="C8" t="s">
         <v>25</v>
-      </c>
-      <c r="E8" t="s" s="43">
-        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -871,8 +836,8 @@
   <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="24.0"/>
-    <col min="2" max="2" customWidth="true" width="25.42578125"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="25.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -884,122 +849,122 @@
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>29</v>
       </c>
-      <c r="B2" s="0">
+      <c r="B2">
         <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="0">
+      <c r="B3">
         <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="0">
+      <c r="B4">
         <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s">
         <v>31</v>
       </c>
-      <c r="B5" s="0">
+      <c r="B5">
         <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" t="s" s="0">
+      <c r="A6" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="0">
+      <c r="B6">
         <v>89</v>
       </c>
     </row>
     <row r="7" spans="1:2">
-      <c r="A7" t="s" s="0">
+      <c r="A7" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="0">
+      <c r="B7">
         <v>90</v>
       </c>
     </row>
     <row r="8" spans="1:2">
-      <c r="A8" t="s" s="0">
+      <c r="A8" t="s">
         <v>34</v>
       </c>
-      <c r="B8" s="0">
+      <c r="B8">
         <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:2">
-      <c r="A9" t="s" s="0">
+      <c r="A9" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="0">
+      <c r="B9">
         <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:2">
-      <c r="A10" t="s" s="0">
+      <c r="A10" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="0">
+      <c r="B10">
         <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:2">
-      <c r="A11" t="s" s="0">
+      <c r="A11" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="0">
+      <c r="B11">
         <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:2">
-      <c r="A12" t="s" s="0">
+      <c r="A12" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="0">
+      <c r="B12">
         <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:2">
-      <c r="A13" t="s" s="0">
+      <c r="A13" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="0">
+      <c r="B13">
         <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:2">
-      <c r="A14" t="s" s="0">
+      <c r="A14" t="s">
         <v>40</v>
       </c>
-      <c r="B14" s="0">
+      <c r="B14">
         <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:2">
-      <c r="A15" t="s" s="0">
+      <c r="A15" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="0">
+      <c r="B15">
         <v>65</v>
       </c>
     </row>
     <row r="16" spans="1:2">
-      <c r="A16" t="s" s="0">
+      <c r="A16" t="s">
         <v>42</v>
       </c>
-      <c r="B16" s="0">
+      <c r="B16">
         <v>66</v>
       </c>
     </row>
@@ -1013,8 +978,8 @@
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="18.5703125"/>
-    <col min="2" max="2" customWidth="true" width="24.42578125"/>
+    <col min="1" max="1" width="18.5703125" customWidth="1"/>
+    <col min="2" max="2" width="24.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="15.75">
@@ -1026,43 +991,116 @@
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>45</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>47</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="4" spans="1:2">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>49</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:2">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s">
         <v>51</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="B5" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:2">
-      <c r="A6" t="s" s="0">
+      <c r="A6" t="s">
         <v>53</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="B6" t="s">
         <v>54</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D76DD3E-E516-4CF3-BDED-A999B55EC4FE}">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="29.7109375" customWidth="1"/>
+    <col min="2" max="2" width="28.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ManageGifts first testcase not completed
</commit_message>
<xml_diff>
--- a/testData/testdata.xlsx
+++ b/testData/testdata.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28723"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28724"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0CE7046C-B6F7-4966-9497-6A697DF6BA80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0F168D41-8420-446D-826A-26218800ED8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" firstSheet="5" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -14,6 +14,7 @@
     <sheet name="Badges " sheetId="4" r:id="rId4"/>
     <sheet name="Earn" sheetId="5" r:id="rId5"/>
     <sheet name="pointsDistributionFilterNames" sheetId="6" r:id="rId6"/>
+    <sheet name="ManageGiftCategory" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="78">
   <si>
     <t>Product Name</t>
   </si>
@@ -240,6 +241,36 @@
   </si>
   <si>
     <t>SALESFORCE</t>
+  </si>
+  <si>
+    <t>Categories</t>
+  </si>
+  <si>
+    <t>Books</t>
+  </si>
+  <si>
+    <t>Clothing</t>
+  </si>
+  <si>
+    <t>Electronics</t>
+  </si>
+  <si>
+    <t>Health and Fitness</t>
+  </si>
+  <si>
+    <t>Stationary</t>
+  </si>
+  <si>
+    <t>Organic Store</t>
+  </si>
+  <si>
+    <t>eVouchers</t>
+  </si>
+  <si>
+    <t>Plants</t>
+  </si>
+  <si>
+    <t>Home Appliance</t>
   </si>
 </sst>
 </file>
@@ -1106,4 +1137,67 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C03319C8-A922-42B5-8644-C9BF6E11F93A}">
+  <dimension ref="A1:A10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="25.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" t="s">
+        <v>77</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>